<commit_message>
updated report, pdf and output map
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valer\Desktop\Replication\JPEtemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB33E967-5C5B-40DF-8BB4-DF01A497BB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="29">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -45,7 +45,73 @@
     <t>Line Number</t>
   </si>
   <si>
-    <t>In-text numbers</t>
+    <t>?</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Reshaped.dta</t>
+  </si>
+  <si>
+    <t>parent_child_PSID.dta</t>
+  </si>
+  <si>
+    <t>Minimal_PSID.dta</t>
+  </si>
+  <si>
+    <t>Income_raw.dta</t>
+  </si>
+  <si>
+    <t>Income_clean.dta</t>
+  </si>
+  <si>
+    <t>Gid_pro_raw.dta</t>
+  </si>
+  <si>
+    <t>Gid_pro_clean.dta</t>
+  </si>
+  <si>
+    <t>Earnings_raw.dta</t>
+  </si>
+  <si>
+    <t>Earnings_clean.dta</t>
+  </si>
+  <si>
+    <t>BLS_CPI_2023.dta</t>
+  </si>
+  <si>
+    <t>pill_by_state.png</t>
+  </si>
+  <si>
+    <t>Pill_IV.do</t>
+  </si>
+  <si>
+    <t>line: 360</t>
+  </si>
+  <si>
+    <t>Table1_covariates.tex</t>
+  </si>
+  <si>
+    <t>Regressions.do</t>
+  </si>
+  <si>
+    <t>Table2_covariates.tex</t>
+  </si>
+  <si>
+    <t>Table3_covariates.tex</t>
+  </si>
+  <si>
+    <t>lines: 1248-1308</t>
+  </si>
+  <si>
+    <t>Table_Educ_1.tex</t>
+  </si>
+  <si>
+    <t>Table_Educ_2.tex</t>
+  </si>
+  <si>
+    <t>lines:1339-1397</t>
   </si>
 </sst>
 </file>
@@ -434,22 +500,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.54296875" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -460,49 +527,223 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
-      </c>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>